<commit_message>
Fix broken trigger reference in example sheet
</commit_message>
<xml_diff>
--- a/tests/workbooktests/workbooks/extras/example_interest_rate_derivatives.xlsx
+++ b/tests/workbooktests/workbooks/extras/example_interest_rate_derivatives.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sebastian\01_GitHub\sschlenkrich\QuantLibXlOil\tests\workbooktests\workbooks\extras\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60A9D16E-ED64-4C10-81AA-C26CA49BC656}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79F2D3D5-8C76-487D-BB21-0CACA6ABA387}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3510" yWindow="-20910" windowWidth="30720" windowHeight="18345" xr2:uid="{E29E0D93-B81D-4342-8E54-9A3C89952B2B}"/>
+    <workbookView xWindow="-120" yWindow="-21720" windowWidth="38640" windowHeight="21120" activeTab="4" xr2:uid="{E29E0D93-B81D-4342-8E54-9A3C89952B2B}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="5" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -598,10 +598,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="4">
-    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd;@"/>
-    <numFmt numFmtId="167" formatCode="0.000%"/>
-    <numFmt numFmtId="169" formatCode="0.00000%"/>
-    <numFmt numFmtId="174" formatCode="0.000"/>
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
+    <numFmt numFmtId="165" formatCode="0.000%"/>
+    <numFmt numFmtId="166" formatCode="0.00000%"/>
+    <numFmt numFmtId="167" formatCode="0.000"/>
   </numFmts>
   <fonts count="9" x14ac:knownFonts="1">
     <font>
@@ -865,8 +865,8 @@
   </cellStyleXfs>
   <cellXfs count="124">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -874,16 +874,16 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="167" fontId="5" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="174" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="167" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="3" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="4" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -909,28 +909,28 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="5" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="5" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="5" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -944,30 +944,30 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="5" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -985,7 +985,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1023,7 +1023,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="2" fontId="5" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="2" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2790,7 +2790,7 @@
         <v>27</v>
       </c>
       <c r="E80" s="57">
-        <f>I58</f>
+        <f t="shared" ref="E80:E87" si="1">I58</f>
         <v>46541</v>
       </c>
       <c r="F80" s="58" cm="1">
@@ -2798,7 +2798,7 @@
         <v>3.4626291513237539E-2</v>
       </c>
       <c r="G80" s="50">
-        <f>F80-M58</f>
+        <f t="shared" ref="G80:G87" si="2">F80-M58</f>
         <v>3.4992565426167632E-2</v>
       </c>
     </row>
@@ -2811,7 +2811,7 @@
         <v>欣[example_interest_rate_derivatives.xlsx]Curves!R81C3YieldTermStructureHandle,A</v>
       </c>
       <c r="E81" s="57">
-        <f>I59</f>
+        <f t="shared" si="1"/>
         <v>46909</v>
       </c>
       <c r="F81" s="58" cm="1">
@@ -2819,13 +2819,13 @@
         <v>3.2256655936068857E-2</v>
       </c>
       <c r="G81" s="50">
-        <f>F81-M59</f>
+        <f t="shared" si="2"/>
         <v>3.2622728461463968E-2</v>
       </c>
     </row>
     <row r="82" spans="2:7" x14ac:dyDescent="0.3">
       <c r="E82" s="57">
-        <f>I60</f>
+        <f t="shared" si="1"/>
         <v>47273</v>
       </c>
       <c r="F82" s="58" cm="1">
@@ -2833,13 +2833,13 @@
         <v>3.1464068845243616E-2</v>
       </c>
       <c r="G82" s="50">
-        <f>F82-M60</f>
+        <f t="shared" si="2"/>
         <v>3.1829990343795286E-2</v>
       </c>
     </row>
     <row r="83" spans="2:7" x14ac:dyDescent="0.3">
       <c r="E83" s="57">
-        <f>I61</f>
+        <f t="shared" si="1"/>
         <v>47637</v>
       </c>
       <c r="F83" s="58" cm="1">
@@ -2847,13 +2847,13 @@
         <v>3.1242194026496625E-2</v>
       </c>
       <c r="G83" s="50">
-        <f>F83-M61</f>
+        <f t="shared" si="2"/>
         <v>3.160802477575924E-2</v>
       </c>
     </row>
     <row r="84" spans="2:7" x14ac:dyDescent="0.3">
       <c r="E84" s="57">
-        <f>I62</f>
+        <f t="shared" si="1"/>
         <v>48002</v>
       </c>
       <c r="F84" s="58" cm="1">
@@ -2861,13 +2861,13 @@
         <v>3.1174868169091315E-2</v>
       </c>
       <c r="G84" s="50">
-        <f>F84-M62</f>
+        <f t="shared" si="2"/>
         <v>3.1540626154044252E-2</v>
       </c>
     </row>
     <row r="85" spans="2:7" x14ac:dyDescent="0.3">
       <c r="E85" s="57">
-        <f>I63</f>
+        <f t="shared" si="1"/>
         <v>48733</v>
       </c>
       <c r="F85" s="58" cm="1">
@@ -2875,13 +2875,13 @@
         <v>3.1207428136625949E-2</v>
       </c>
       <c r="G85" s="50">
-        <f>F85-M63</f>
+        <f t="shared" si="2"/>
         <v>3.157307475477826E-2</v>
       </c>
     </row>
     <row r="86" spans="2:7" x14ac:dyDescent="0.3">
       <c r="E86" s="57">
-        <f>I64</f>
+        <f t="shared" si="1"/>
         <v>49829</v>
       </c>
       <c r="F86" s="58" cm="1">
@@ -2889,13 +2889,13 @@
         <v>3.1186666702453285E-2</v>
       </c>
       <c r="G86" s="50">
-        <f>F86-M64</f>
+        <f t="shared" si="2"/>
         <v>3.1552199179489759E-2</v>
       </c>
     </row>
     <row r="87" spans="2:7" x14ac:dyDescent="0.3">
       <c r="E87" s="59">
-        <f>I65</f>
+        <f t="shared" si="1"/>
         <v>50559</v>
       </c>
       <c r="F87" s="60" cm="1">
@@ -2903,7 +2903,7 @@
         <v>3.1052022548249434E-2</v>
       </c>
       <c r="G87" s="51">
-        <f>F87-M65</f>
+        <f t="shared" si="2"/>
         <v>3.1417509540039565E-2</v>
       </c>
     </row>
@@ -6936,7 +6936,7 @@
         <v>97</v>
       </c>
       <c r="F17" s="27" cm="1">
-        <f t="array" ref="F17">_xll.qlCalendarAdvance("NYC",_xll.qlCalendarAdvance("NYC",$C$16,E17),"-2d","Preceding",,C2)</f>
+        <f t="array" ref="F17">_xll.qlCalendarAdvance("NYC",_xll.qlCalendarAdvance("NYC",$C$16,E17),"-2d","Preceding",,$C$2)</f>
         <v>46510</v>
       </c>
       <c r="G17" s="27" cm="1">
@@ -6960,7 +6960,7 @@
         <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R17C11EuropeanExercise,A</v>
       </c>
       <c r="L17" s="26" t="str" cm="1">
-        <f t="array" ref="L17">_xll.qlSwaption(I17,K17,,,C2)</f>
+        <f t="array" ref="L17">_xll.qlSwaption(I17,K17,,,$C$2)</f>
         <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R17C12Swaption,A</v>
       </c>
       <c r="M17" s="88" cm="1">
@@ -6980,7 +6980,7 @@
         <v>6.8192074362781394E-3</v>
       </c>
       <c r="R17" s="112">
-        <f>G17-F17</f>
+        <f t="shared" ref="R17:R25" si="0">G17-F17</f>
         <v>2</v>
       </c>
       <c r="S17" s="113" t="str">
@@ -6988,14 +6988,14 @@
         <v>9y</v>
       </c>
       <c r="T17" s="26" t="str" cm="1">
-        <f t="array" ref="T17">_xll.qlSwaptionHelper(F17,S17,Q17,$C$19,"3m","Act/360","Act/360",$C$4,,$C$22,,"Normal",,R17,"Compound",C2)</f>
+        <f t="array" ref="T17">_xll.qlSwaptionHelper(F17,S17,Q17,$C$19,"3m","Act/360","Act/360",$C$4,,$C$22,,"Normal",,R17,"Compound",$C$2)</f>
         <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R17C20SwaptionHelper,A</v>
       </c>
       <c r="U17" s="68">
         <v>7.0000000000000001E-3</v>
       </c>
       <c r="V17" s="114">
-        <f>$C$30</f>
+        <f t="shared" ref="V17:V26" si="1">$C$30</f>
         <v>0.01</v>
       </c>
       <c r="W17" s="115" t="b" cm="1">
@@ -7019,7 +7019,7 @@
         <v>98</v>
       </c>
       <c r="F18" s="32" cm="1">
-        <f t="array" ref="F18">_xll.qlCalendarAdvance("NYC",_xll.qlCalendarAdvance("NYC",$C$16,E18),"-2d","Preceding",,C3)</f>
+        <f t="array" ref="F18">_xll.qlCalendarAdvance("NYC",_xll.qlCalendarAdvance("NYC",$C$16,E18),"-2d","Preceding",,$C$2)</f>
         <v>46876</v>
       </c>
       <c r="G18" s="32" cm="1">
@@ -7043,7 +7043,7 @@
         <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R18C11EuropeanExercise,A</v>
       </c>
       <c r="L18" s="31" t="str" cm="1">
-        <f t="array" ref="L18">_xll.qlSwaption(I18,K18,,,C3)</f>
+        <f t="array" ref="L18">_xll.qlSwaption(I18,K18,,,$C$2)</f>
         <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R18C12Swaption,A</v>
       </c>
       <c r="M18" s="90" cm="1">
@@ -7063,22 +7063,22 @@
         <v>6.8439003518695187E-3</v>
       </c>
       <c r="R18" s="116">
-        <f>G18-F18</f>
+        <f t="shared" si="0"/>
         <v>2</v>
       </c>
       <c r="S18" s="117" t="str">
-        <f t="shared" ref="S18:S25" si="0">ROUND(($C$17-G18)/365.25,0)&amp;"y"</f>
+        <f t="shared" ref="S18:S25" si="2">ROUND(($C$17-G18)/365.25,0)&amp;"y"</f>
         <v>8y</v>
       </c>
       <c r="T18" s="31" t="str" cm="1">
-        <f t="array" ref="T18">_xll.qlSwaptionHelper(F18,S18,Q18,$C$19,"3m","Act/360","Act/360",$C$4,,$C$22,,"Normal",,R18,"Compound",C3)</f>
+        <f t="array" ref="T18">_xll.qlSwaptionHelper(F18,S18,Q18,$C$19,"3m","Act/360","Act/360",$C$4,,$C$22,,"Normal",,R18,"Compound",$C$2)</f>
         <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R18C20SwaptionHelper,A</v>
       </c>
       <c r="U18" s="69">
         <v>7.0000000000000001E-3</v>
       </c>
       <c r="V18" s="118">
-        <f>$C$30</f>
+        <f t="shared" si="1"/>
         <v>0.01</v>
       </c>
       <c r="W18" s="63" t="b" cm="1">
@@ -7101,7 +7101,7 @@
         <v>99</v>
       </c>
       <c r="F19" s="32" cm="1">
-        <f t="array" ref="F19">_xll.qlCalendarAdvance("NYC",_xll.qlCalendarAdvance("NYC",$C$16,E19),"-2d","Preceding",,C4)</f>
+        <f t="array" ref="F19">_xll.qlCalendarAdvance("NYC",_xll.qlCalendarAdvance("NYC",$C$16,E19),"-2d","Preceding",,$C$2)</f>
         <v>47241</v>
       </c>
       <c r="G19" s="32" cm="1">
@@ -7125,7 +7125,7 @@
         <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R19C11EuropeanExercise,A</v>
       </c>
       <c r="L19" s="31" t="str" cm="1">
-        <f t="array" ref="L19">_xll.qlSwaption(I19,K19,,,C4)</f>
+        <f t="array" ref="L19">_xll.qlSwaption(I19,K19,,,$C$2)</f>
         <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R19C12Swaption,A</v>
       </c>
       <c r="M19" s="90" cm="1">
@@ -7145,22 +7145,22 @@
         <v>6.8685932674608981E-3</v>
       </c>
       <c r="R19" s="116">
-        <f>G19-F19</f>
+        <f t="shared" si="0"/>
         <v>4</v>
       </c>
       <c r="S19" s="117" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>7y</v>
       </c>
       <c r="T19" s="31" t="str" cm="1">
-        <f t="array" ref="T19">_xll.qlSwaptionHelper(F19,S19,Q19,$C$19,"3m","Act/360","Act/360",$C$4,,$C$22,,"Normal",,R19,"Compound",C4)</f>
+        <f t="array" ref="T19">_xll.qlSwaptionHelper(F19,S19,Q19,$C$19,"3m","Act/360","Act/360",$C$4,,$C$22,,"Normal",,R19,"Compound",$C$2)</f>
         <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R19C20SwaptionHelper,A</v>
       </c>
       <c r="U19" s="69">
         <v>7.0000000000000001E-3</v>
       </c>
       <c r="V19" s="118">
-        <f>$C$30</f>
+        <f t="shared" si="1"/>
         <v>0.01</v>
       </c>
       <c r="W19" s="63" t="b" cm="1">
@@ -7176,7 +7176,7 @@
         <v>104</v>
       </c>
       <c r="F20" s="32" cm="1">
-        <f t="array" ref="F20">_xll.qlCalendarAdvance("NYC",_xll.qlCalendarAdvance("NYC",$C$16,E20),"-2d","Preceding",,C5)</f>
+        <f t="array" ref="F20">_xll.qlCalendarAdvance("NYC",_xll.qlCalendarAdvance("NYC",$C$16,E20),"-2d","Preceding",,$C$2)</f>
         <v>47605</v>
       </c>
       <c r="G20" s="32" cm="1">
@@ -7200,7 +7200,7 @@
         <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R20C11EuropeanExercise,A</v>
       </c>
       <c r="L20" s="31" t="str" cm="1">
-        <f t="array" ref="L20">_xll.qlSwaption(I20,K20,,,C5)</f>
+        <f t="array" ref="L20">_xll.qlSwaption(I20,K20,,,$C$2)</f>
         <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R20C12Swaption,A</v>
       </c>
       <c r="M20" s="90" cm="1">
@@ -7220,22 +7220,22 @@
         <v>6.8710196098611381E-3</v>
       </c>
       <c r="R20" s="116">
-        <f>G20-F20</f>
+        <f t="shared" si="0"/>
         <v>4</v>
       </c>
       <c r="S20" s="117" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>6y</v>
       </c>
       <c r="T20" s="31" t="str" cm="1">
-        <f t="array" ref="T20">_xll.qlSwaptionHelper(F20,S20,Q20,$C$19,"3m","Act/360","Act/360",$C$4,,$C$22,,"Normal",,R20,"Compound",#REF!)</f>
+        <f t="array" ref="T20">_xll.qlSwaptionHelper(F20,S20,Q20,$C$19,"3m","Act/360","Act/360",$C$4,,$C$22,,"Normal",,R20,"Compound",$C$2)</f>
         <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R20C20SwaptionHelper,A</v>
       </c>
       <c r="U20" s="69">
         <v>7.0000000000000001E-3</v>
       </c>
       <c r="V20" s="118">
-        <f>$C$30</f>
+        <f t="shared" si="1"/>
         <v>0.01</v>
       </c>
       <c r="W20" s="63" t="b" cm="1">
@@ -7257,7 +7257,7 @@
         <v>100</v>
       </c>
       <c r="F21" s="32" cm="1">
-        <f t="array" ref="F21">_xll.qlCalendarAdvance("NYC",_xll.qlCalendarAdvance("NYC",$C$16,E21),"-2d","Preceding",,C6)</f>
+        <f t="array" ref="F21">_xll.qlCalendarAdvance("NYC",_xll.qlCalendarAdvance("NYC",$C$16,E21),"-2d","Preceding",,$C$2)</f>
         <v>47969</v>
       </c>
       <c r="G21" s="32" cm="1">
@@ -7281,7 +7281,7 @@
         <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R21C11EuropeanExercise,A</v>
       </c>
       <c r="L21" s="31" t="str" cm="1">
-        <f t="array" ref="L21">_xll.qlSwaption(I21,K21,,,C6)</f>
+        <f t="array" ref="L21">_xll.qlSwaption(I21,K21,,,$C$2)</f>
         <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R21C12Swaption,A</v>
       </c>
       <c r="M21" s="90" cm="1">
@@ -7301,22 +7301,22 @@
         <v>6.8386420675278876E-3</v>
       </c>
       <c r="R21" s="116">
-        <f>G21-F21</f>
+        <f t="shared" si="0"/>
         <v>4</v>
       </c>
       <c r="S21" s="117" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>5y</v>
       </c>
       <c r="T21" s="31" t="str" cm="1">
-        <f t="array" ref="T21">_xll.qlSwaptionHelper(F21,S21,Q21,$C$19,"3m","Act/360","Act/360",$C$4,,$C$22,,"Normal",,R21,"Compound",C5)</f>
+        <f t="array" ref="T21">_xll.qlSwaptionHelper(F21,S21,Q21,$C$19,"3m","Act/360","Act/360",$C$4,,$C$22,,"Normal",,R21,"Compound",$C$2)</f>
         <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R21C20SwaptionHelper,A</v>
       </c>
       <c r="U21" s="69">
         <v>7.0000000000000001E-3</v>
       </c>
       <c r="V21" s="118">
-        <f>$C$30</f>
+        <f t="shared" si="1"/>
         <v>0.01</v>
       </c>
       <c r="W21" s="63" t="b" cm="1">
@@ -7338,7 +7338,7 @@
         <v>105</v>
       </c>
       <c r="F22" s="32" cm="1">
-        <f t="array" ref="F22">_xll.qlCalendarAdvance("NYC",_xll.qlCalendarAdvance("NYC",$C$16,E22),"-2d","Preceding",,C7)</f>
+        <f t="array" ref="F22">_xll.qlCalendarAdvance("NYC",_xll.qlCalendarAdvance("NYC",$C$16,E22),"-2d","Preceding",,$C$2)</f>
         <v>48337</v>
       </c>
       <c r="G22" s="32" cm="1">
@@ -7362,7 +7362,7 @@
         <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R22C11EuropeanExercise,A</v>
       </c>
       <c r="L22" s="31" t="str" cm="1">
-        <f t="array" ref="L22">_xll.qlSwaption(I22,K22,,,C7)</f>
+        <f t="array" ref="L22">_xll.qlSwaption(I22,K22,,,$C$2)</f>
         <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R22C12Swaption,A</v>
       </c>
       <c r="M22" s="90" cm="1">
@@ -7382,22 +7382,22 @@
         <v>6.8094752901471274E-3</v>
       </c>
       <c r="R22" s="116">
-        <f>G22-F22</f>
+        <f t="shared" si="0"/>
         <v>2</v>
       </c>
       <c r="S22" s="117" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>4y</v>
       </c>
       <c r="T22" s="31" t="str" cm="1">
-        <f t="array" ref="T22">_xll.qlSwaptionHelper(F22,S22,Q22,$C$19,"3m","Act/360","Act/360",$C$4,,$C$22,,"Normal",,R22,"Compound",#REF!)</f>
+        <f t="array" ref="T22">_xll.qlSwaptionHelper(F22,S22,Q22,$C$19,"3m","Act/360","Act/360",$C$4,,$C$22,,"Normal",,R22,"Compound",$C$2)</f>
         <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R22C20SwaptionHelper,A</v>
       </c>
       <c r="U22" s="69">
         <v>7.0000000000000001E-3</v>
       </c>
       <c r="V22" s="118">
-        <f>$C$30</f>
+        <f t="shared" si="1"/>
         <v>0.01</v>
       </c>
       <c r="W22" s="63" t="b" cm="1">
@@ -7413,7 +7413,7 @@
         <v>101</v>
       </c>
       <c r="F23" s="32" cm="1">
-        <f t="array" ref="F23">_xll.qlCalendarAdvance("NYC",_xll.qlCalendarAdvance("NYC",$C$16,E23),"-2d","Preceding",,C8)</f>
+        <f t="array" ref="F23">_xll.qlCalendarAdvance("NYC",_xll.qlCalendarAdvance("NYC",$C$16,E23),"-2d","Preceding",,$C$2)</f>
         <v>48702</v>
       </c>
       <c r="G23" s="32" cm="1">
@@ -7437,7 +7437,7 @@
         <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R23C11EuropeanExercise,A</v>
       </c>
       <c r="L23" s="31" t="str" cm="1">
-        <f t="array" ref="L23">_xll.qlSwaption(I23,K23,,,C8)</f>
+        <f t="array" ref="L23">_xll.qlSwaption(I23,K23,,,$C$2)</f>
         <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R23C12Swaption,A</v>
       </c>
       <c r="M23" s="90" cm="1">
@@ -7457,22 +7457,22 @@
         <v>6.7899775764584816E-3</v>
       </c>
       <c r="R23" s="116">
-        <f>G23-F23</f>
+        <f t="shared" si="0"/>
         <v>2</v>
       </c>
       <c r="S23" s="117" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>3y</v>
       </c>
       <c r="T23" s="31" t="str" cm="1">
-        <f t="array" ref="T23">_xll.qlSwaptionHelper(F23,S23,Q23,$C$19,"3m","Act/360","Act/360",$C$4,,$C$22,,"Normal",,R23,"Compound",C6)</f>
+        <f t="array" ref="T23">_xll.qlSwaptionHelper(F23,S23,Q23,$C$19,"3m","Act/360","Act/360",$C$4,,$C$22,,"Normal",,R23,"Compound",$C$2)</f>
         <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R23C20SwaptionHelper,A</v>
       </c>
       <c r="U23" s="69">
         <v>7.0000000000000001E-3</v>
       </c>
       <c r="V23" s="118">
-        <f>$C$30</f>
+        <f t="shared" si="1"/>
         <v>0.01</v>
       </c>
       <c r="W23" s="63" t="b" cm="1">
@@ -7488,7 +7488,7 @@
         <v>106</v>
       </c>
       <c r="F24" s="32" cm="1">
-        <f t="array" ref="F24">_xll.qlCalendarAdvance("NYC",_xll.qlCalendarAdvance("NYC",$C$16,E24),"-2d","Preceding",,C9)</f>
+        <f t="array" ref="F24">_xll.qlCalendarAdvance("NYC",_xll.qlCalendarAdvance("NYC",$C$16,E24),"-2d","Preceding",,$C$2)</f>
         <v>49067</v>
       </c>
       <c r="G24" s="32" cm="1">
@@ -7512,7 +7512,7 @@
         <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R24C11EuropeanExercise,A</v>
       </c>
       <c r="L24" s="31" t="str" cm="1">
-        <f t="array" ref="L24">_xll.qlSwaption(I24,K24,,,C9)</f>
+        <f t="array" ref="L24">_xll.qlSwaption(I24,K24,,,$C$2)</f>
         <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R24C12Swaption,A</v>
       </c>
       <c r="M24" s="90" cm="1">
@@ -7532,22 +7532,22 @@
         <v>6.8705740176875649E-3</v>
       </c>
       <c r="R24" s="116">
-        <f>G24-F24</f>
+        <f t="shared" si="0"/>
         <v>2</v>
       </c>
       <c r="S24" s="117" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>2y</v>
       </c>
       <c r="T24" s="31" t="str" cm="1">
-        <f t="array" ref="T24">_xll.qlSwaptionHelper(F24,S24,Q24,$C$19,"3m","Act/360","Act/360",$C$4,,$C$22,,"Normal",,R24,"Compound",C7)</f>
+        <f t="array" ref="T24">_xll.qlSwaptionHelper(F24,S24,Q24,$C$19,"3m","Act/360","Act/360",$C$4,,$C$22,,"Normal",,R24,"Compound",$C$2)</f>
         <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R24C20SwaptionHelper,A</v>
       </c>
       <c r="U24" s="69">
         <v>7.0000000000000001E-3</v>
       </c>
       <c r="V24" s="118">
-        <f>$C$30</f>
+        <f t="shared" si="1"/>
         <v>0.01</v>
       </c>
       <c r="W24" s="63" t="b" cm="1">
@@ -7563,7 +7563,7 @@
         <v>107</v>
       </c>
       <c r="F25" s="37" cm="1">
-        <f t="array" ref="F25">_xll.qlCalendarAdvance("NYC",_xll.qlCalendarAdvance("NYC",$C$16,E25),"-2d","Preceding",,C10)</f>
+        <f t="array" ref="F25">_xll.qlCalendarAdvance("NYC",_xll.qlCalendarAdvance("NYC",$C$16,E25),"-2d","Preceding",,$C$2)</f>
         <v>49432</v>
       </c>
       <c r="G25" s="37" cm="1">
@@ -7587,7 +7587,7 @@
         <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R25C11EuropeanExercise,A</v>
       </c>
       <c r="L25" s="36" t="str" cm="1">
-        <f t="array" ref="L25">_xll.qlSwaption(I25,K25,,,C10)</f>
+        <f t="array" ref="L25">_xll.qlSwaption(I25,K25,,,$C$2)</f>
         <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R25C12Swaption,A</v>
       </c>
       <c r="M25" s="92" cm="1">
@@ -7607,22 +7607,22 @@
         <v>6.7898728295167242E-3</v>
       </c>
       <c r="R25" s="116">
-        <f>G25-F25</f>
+        <f t="shared" si="0"/>
         <v>4</v>
       </c>
       <c r="S25" s="117" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>1y</v>
       </c>
       <c r="T25" s="31" t="str" cm="1">
-        <f t="array" ref="T25">_xll.qlSwaptionHelper(F25,S25,Q25,$C$19,"3m","Act/360","Act/360",$C$4,,$C$22,,"Normal",,R25,"Compound",C8)</f>
+        <f t="array" ref="T25">_xll.qlSwaptionHelper(F25,S25,Q25,$C$19,"3m","Act/360","Act/360",$C$4,,$C$22,,"Normal",,R25,"Compound",$C$2)</f>
         <v>欣[example_interest_rate_derivatives.xlsx]Swaptions!R25C20SwaptionHelper,A</v>
       </c>
       <c r="U25" s="69">
         <v>7.0000000000000001E-3</v>
       </c>
       <c r="V25" s="118">
-        <f>$C$30</f>
+        <f t="shared" si="1"/>
         <v>0.01</v>
       </c>
       <c r="W25" s="63" t="b" cm="1">
@@ -7642,7 +7642,7 @@
         <v>7.0000000000000001E-3</v>
       </c>
       <c r="V26" s="120">
-        <f>$C$30</f>
+        <f t="shared" si="1"/>
         <v>0.01</v>
       </c>
       <c r="W26" s="39"/>
@@ -7798,7 +7798,7 @@
     </row>
     <row r="53" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B53" s="87" t="str">
-        <f>E17&amp;"-"&amp;S17</f>
+        <f t="shared" ref="B53:B61" si="3">E17&amp;"-"&amp;S17</f>
         <v>1y-9y</v>
       </c>
       <c r="C53" s="88" cm="1">
@@ -7812,7 +7812,7 @@
     </row>
     <row r="54" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B54" s="89" t="str">
-        <f>E18&amp;"-"&amp;S18</f>
+        <f t="shared" si="3"/>
         <v>2y-8y</v>
       </c>
       <c r="C54" s="90" cm="1">
@@ -7826,7 +7826,7 @@
     </row>
     <row r="55" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B55" s="89" t="str">
-        <f>E19&amp;"-"&amp;S19</f>
+        <f t="shared" si="3"/>
         <v>3y-7y</v>
       </c>
       <c r="C55" s="90" cm="1">
@@ -7840,7 +7840,7 @@
     </row>
     <row r="56" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B56" s="89" t="str">
-        <f>E20&amp;"-"&amp;S20</f>
+        <f t="shared" si="3"/>
         <v>4y-6y</v>
       </c>
       <c r="C56" s="90" cm="1">
@@ -7854,7 +7854,7 @@
     </row>
     <row r="57" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B57" s="89" t="str">
-        <f>E21&amp;"-"&amp;S21</f>
+        <f t="shared" si="3"/>
         <v>5y-5y</v>
       </c>
       <c r="C57" s="90" cm="1">
@@ -7868,7 +7868,7 @@
     </row>
     <row r="58" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B58" s="89" t="str">
-        <f>E22&amp;"-"&amp;S22</f>
+        <f t="shared" si="3"/>
         <v>6y-4y</v>
       </c>
       <c r="C58" s="90" cm="1">
@@ -7882,7 +7882,7 @@
     </row>
     <row r="59" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B59" s="89" t="str">
-        <f>E23&amp;"-"&amp;S23</f>
+        <f t="shared" si="3"/>
         <v>7y-3y</v>
       </c>
       <c r="C59" s="90" cm="1">
@@ -7896,7 +7896,7 @@
     </row>
     <row r="60" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B60" s="89" t="str">
-        <f>E24&amp;"-"&amp;S24</f>
+        <f t="shared" si="3"/>
         <v>8y-2y</v>
       </c>
       <c r="C60" s="90" cm="1">
@@ -7910,7 +7910,7 @@
     </row>
     <row r="61" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B61" s="89" t="str">
-        <f>E25&amp;"-"&amp;S25</f>
+        <f t="shared" si="3"/>
         <v>9y-1y</v>
       </c>
       <c r="C61" s="90" cm="1">

</xml_diff>